<commit_message>
Modelle Methane Vervollständigt und Sensitivity umgebaut
</commit_message>
<xml_diff>
--- a/Ammoniak/Ammoniak_Greenfield_Patagonien/Datenbank.xlsx
+++ b/Ammoniak/Ammoniak_Greenfield_Patagonien/Datenbank.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hem38994\Documents\GitHub\FENES_P2X\Ammoniak\Ammoniak_Greenfield_Patagonien\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Ammoniak\Ammoniak_Greenfield_Patagonien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2D360A-E98B-499A-9256-F9FFD0C8BFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA533C9-47B2-4025-8F9A-E15299DAE437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1025,10 +1025,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -1164,20 +1164,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1185,11 +1185,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1202,28 +1202,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1263,43 +1263,43 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1666,7 +1666,7 @@
         <v>28</v>
       </c>
       <c r="E4" s="21">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="F4" t="s">
         <v>101</v>
@@ -2587,10 +2587,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="67" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="70" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28" t="s">
@@ -2605,8 +2605,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="65"/>
-      <c r="B3" s="67"/>
+      <c r="A3" s="68"/>
+      <c r="B3" s="65"/>
       <c r="C3" s="13" t="s">
         <v>135</v>
       </c>
@@ -2619,8 +2619,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="65"/>
-      <c r="B4" s="67"/>
+      <c r="A4" s="68"/>
+      <c r="B4" s="65"/>
       <c r="C4" s="13" t="s">
         <v>102</v>
       </c>
@@ -2633,8 +2633,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="65"/>
-      <c r="B5" s="67"/>
+      <c r="A5" s="68"/>
+      <c r="B5" s="65"/>
       <c r="C5" s="13" t="s">
         <v>171</v>
       </c>
@@ -2647,8 +2647,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="65"/>
-      <c r="B6" s="67"/>
+      <c r="A6" s="68"/>
+      <c r="B6" s="65"/>
       <c r="C6" s="13" t="s">
         <v>183</v>
       </c>
@@ -2661,8 +2661,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="65"/>
-      <c r="B7" s="67"/>
+      <c r="A7" s="68"/>
+      <c r="B7" s="65"/>
       <c r="C7" s="13" t="s">
         <v>201</v>
       </c>
@@ -2675,8 +2675,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="65"/>
-      <c r="B8" s="67"/>
+      <c r="A8" s="68"/>
+      <c r="B8" s="65"/>
       <c r="C8" s="13" t="s">
         <v>249</v>
       </c>
@@ -2689,8 +2689,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="65"/>
-      <c r="B9" s="67"/>
+      <c r="A9" s="68"/>
+      <c r="B9" s="65"/>
       <c r="C9" s="13" t="s">
         <v>215</v>
       </c>
@@ -2703,8 +2703,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="65"/>
-      <c r="B10" s="67"/>
+      <c r="A10" s="68"/>
+      <c r="B10" s="65"/>
       <c r="C10" s="13" t="s">
         <v>239</v>
       </c>
@@ -2717,13 +2717,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="65"/>
-      <c r="B11" s="67"/>
+      <c r="A11" s="68"/>
+      <c r="B11" s="65"/>
       <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="65"/>
-      <c r="B12" s="68" t="s">
+      <c r="A12" s="68"/>
+      <c r="B12" s="64" t="s">
         <v>3</v>
       </c>
       <c r="C12" s="37" t="s">
@@ -2738,8 +2738,8 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="65"/>
-      <c r="B13" s="67"/>
+      <c r="A13" s="68"/>
+      <c r="B13" s="65"/>
       <c r="C13" s="13" t="s">
         <v>176</v>
       </c>
@@ -2752,8 +2752,8 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="65"/>
-      <c r="B14" s="67"/>
+      <c r="A14" s="68"/>
+      <c r="B14" s="65"/>
       <c r="C14" s="13" t="s">
         <v>179</v>
       </c>
@@ -2766,8 +2766,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="65"/>
-      <c r="B15" s="67"/>
+      <c r="A15" s="68"/>
+      <c r="B15" s="65"/>
       <c r="C15" s="13" t="s">
         <v>180</v>
       </c>
@@ -2780,8 +2780,8 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="65"/>
-      <c r="B16" s="67"/>
+      <c r="A16" s="68"/>
+      <c r="B16" s="65"/>
       <c r="C16" s="13" t="s">
         <v>102</v>
       </c>
@@ -2794,8 +2794,8 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="65"/>
-      <c r="B17" s="67"/>
+      <c r="A17" s="68"/>
+      <c r="B17" s="65"/>
       <c r="C17" s="13" t="s">
         <v>183</v>
       </c>
@@ -2808,8 +2808,8 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="65"/>
-      <c r="B18" s="67"/>
+      <c r="A18" s="68"/>
+      <c r="B18" s="65"/>
       <c r="C18" s="13" t="s">
         <v>201</v>
       </c>
@@ -2822,8 +2822,8 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="65"/>
-      <c r="B19" s="67"/>
+      <c r="A19" s="68"/>
+      <c r="B19" s="65"/>
       <c r="C19" s="13" t="s">
         <v>249</v>
       </c>
@@ -2836,8 +2836,8 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="65"/>
-      <c r="B20" s="67"/>
+      <c r="A20" s="68"/>
+      <c r="B20" s="65"/>
       <c r="C20" s="13" t="s">
         <v>215</v>
       </c>
@@ -2850,8 +2850,8 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="65"/>
-      <c r="B21" s="67"/>
+      <c r="A21" s="68"/>
+      <c r="B21" s="65"/>
       <c r="C21" s="13" t="s">
         <v>239</v>
       </c>
@@ -2864,16 +2864,16 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="65"/>
-      <c r="B22" s="69"/>
+      <c r="A22" s="68"/>
+      <c r="B22" s="66"/>
       <c r="C22" s="39"/>
       <c r="D22" s="39"/>
       <c r="E22" s="40"/>
       <c r="F22" s="39"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="65"/>
-      <c r="B23" s="70" t="s">
+      <c r="A23" s="68"/>
+      <c r="B23" s="73" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="13" t="s">
@@ -2888,8 +2888,8 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="65"/>
-      <c r="B24" s="70"/>
+      <c r="A24" s="68"/>
+      <c r="B24" s="73"/>
       <c r="C24" s="13" t="s">
         <v>135</v>
       </c>
@@ -2902,8 +2902,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="65"/>
-      <c r="B25" s="70"/>
+      <c r="A25" s="68"/>
+      <c r="B25" s="73"/>
       <c r="C25" s="13" t="s">
         <v>102</v>
       </c>
@@ -2916,8 +2916,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="65"/>
-      <c r="B26" s="70"/>
+      <c r="A26" s="68"/>
+      <c r="B26" s="73"/>
       <c r="C26" s="13" t="s">
         <v>173</v>
       </c>
@@ -2930,8 +2930,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="65"/>
-      <c r="B27" s="70"/>
+      <c r="A27" s="68"/>
+      <c r="B27" s="73"/>
       <c r="C27" s="13" t="s">
         <v>183</v>
       </c>
@@ -2944,8 +2944,8 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="65"/>
-      <c r="B28" s="70"/>
+      <c r="A28" s="68"/>
+      <c r="B28" s="73"/>
       <c r="C28" s="13" t="s">
         <v>201</v>
       </c>
@@ -2958,8 +2958,8 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="65"/>
-      <c r="B29" s="70"/>
+      <c r="A29" s="68"/>
+      <c r="B29" s="73"/>
       <c r="C29" s="13" t="s">
         <v>249</v>
       </c>
@@ -2972,8 +2972,8 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="65"/>
-      <c r="B30" s="70"/>
+      <c r="A30" s="68"/>
+      <c r="B30" s="73"/>
       <c r="C30" s="13" t="s">
         <v>215</v>
       </c>
@@ -2986,8 +2986,8 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="65"/>
-      <c r="B31" s="70"/>
+      <c r="A31" s="68"/>
+      <c r="B31" s="73"/>
       <c r="C31" s="13" t="s">
         <v>239</v>
       </c>
@@ -3000,15 +3000,15 @@
       </c>
     </row>
     <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="65"/>
-      <c r="B32" s="70"/>
+      <c r="A32" s="68"/>
+      <c r="B32" s="73"/>
       <c r="E32" s="35"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="64" t="s">
+      <c r="A33" s="67" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="72" t="s">
+      <c r="B33" s="76" t="s">
         <v>5</v>
       </c>
       <c r="C33" s="28" t="s">
@@ -3023,8 +3023,8 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="65"/>
-      <c r="B34" s="70"/>
+      <c r="A34" s="68"/>
+      <c r="B34" s="73"/>
       <c r="C34" s="13" t="s">
         <v>139</v>
       </c>
@@ -3037,8 +3037,8 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="65"/>
-      <c r="B35" s="70"/>
+      <c r="A35" s="68"/>
+      <c r="B35" s="73"/>
       <c r="C35" s="13" t="s">
         <v>168</v>
       </c>
@@ -3051,8 +3051,8 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="65"/>
-      <c r="B36" s="70"/>
+      <c r="A36" s="68"/>
+      <c r="B36" s="73"/>
       <c r="C36" s="13" t="s">
         <v>169</v>
       </c>
@@ -3065,8 +3065,8 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="65"/>
-      <c r="B37" s="70"/>
+      <c r="A37" s="68"/>
+      <c r="B37" s="73"/>
       <c r="C37" s="13" t="s">
         <v>183</v>
       </c>
@@ -3079,8 +3079,8 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="65"/>
-      <c r="B38" s="70"/>
+      <c r="A38" s="68"/>
+      <c r="B38" s="73"/>
       <c r="C38" s="13" t="s">
         <v>201</v>
       </c>
@@ -3093,8 +3093,8 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="65"/>
-      <c r="B39" s="70"/>
+      <c r="A39" s="68"/>
+      <c r="B39" s="73"/>
       <c r="C39" s="13" t="s">
         <v>249</v>
       </c>
@@ -3107,8 +3107,8 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="65"/>
-      <c r="B40" s="70"/>
+      <c r="A40" s="68"/>
+      <c r="B40" s="73"/>
       <c r="C40" s="13" t="s">
         <v>215</v>
       </c>
@@ -3121,8 +3121,8 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="65"/>
-      <c r="B41" s="70"/>
+      <c r="A41" s="68"/>
+      <c r="B41" s="73"/>
       <c r="C41" s="13" t="s">
         <v>239</v>
       </c>
@@ -3135,13 +3135,13 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="65"/>
-      <c r="B42" s="70"/>
+      <c r="A42" s="68"/>
+      <c r="B42" s="73"/>
       <c r="E42" s="35"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="65"/>
-      <c r="B43" s="73" t="s">
+      <c r="A43" s="68"/>
+      <c r="B43" s="72" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="37" t="s">
@@ -3156,8 +3156,8 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="65"/>
-      <c r="B44" s="70"/>
+      <c r="A44" s="68"/>
+      <c r="B44" s="73"/>
       <c r="C44" s="13" t="s">
         <v>141</v>
       </c>
@@ -3170,8 +3170,8 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="65"/>
-      <c r="B45" s="67"/>
+      <c r="A45" s="68"/>
+      <c r="B45" s="65"/>
       <c r="C45" s="13" t="s">
         <v>139</v>
       </c>
@@ -3184,8 +3184,8 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="65"/>
-      <c r="B46" s="67"/>
+      <c r="A46" s="68"/>
+      <c r="B46" s="65"/>
       <c r="C46" s="13" t="s">
         <v>135</v>
       </c>
@@ -3198,8 +3198,8 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="65"/>
-      <c r="B47" s="67"/>
+      <c r="A47" s="68"/>
+      <c r="B47" s="65"/>
       <c r="C47" s="13" t="s">
         <v>156</v>
       </c>
@@ -3212,8 +3212,8 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="65"/>
-      <c r="B48" s="67"/>
+      <c r="A48" s="68"/>
+      <c r="B48" s="65"/>
       <c r="C48" s="13" t="s">
         <v>157</v>
       </c>
@@ -3226,8 +3226,8 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="65"/>
-      <c r="B49" s="67"/>
+      <c r="A49" s="68"/>
+      <c r="B49" s="65"/>
       <c r="C49" s="13" t="s">
         <v>183</v>
       </c>
@@ -3240,8 +3240,8 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="65"/>
-      <c r="B50" s="67"/>
+      <c r="A50" s="68"/>
+      <c r="B50" s="65"/>
       <c r="C50" s="13" t="s">
         <v>201</v>
       </c>
@@ -3254,8 +3254,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="65"/>
-      <c r="B51" s="67"/>
+      <c r="A51" s="68"/>
+      <c r="B51" s="65"/>
       <c r="C51" s="13" t="s">
         <v>249</v>
       </c>
@@ -3268,8 +3268,8 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="65"/>
-      <c r="B52" s="67"/>
+      <c r="A52" s="68"/>
+      <c r="B52" s="65"/>
       <c r="C52" s="13" t="s">
         <v>215</v>
       </c>
@@ -3282,8 +3282,8 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="65"/>
-      <c r="B53" s="67"/>
+      <c r="A53" s="68"/>
+      <c r="B53" s="65"/>
       <c r="C53" s="13" t="s">
         <v>239</v>
       </c>
@@ -3297,17 +3297,17 @@
     </row>
     <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="71"/>
-      <c r="B54" s="74"/>
+      <c r="B54" s="69"/>
       <c r="C54" s="43"/>
       <c r="D54" s="43"/>
       <c r="E54" s="44"/>
       <c r="F54" s="43"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="64" t="s">
+      <c r="A55" s="67" t="s">
         <v>86</v>
       </c>
-      <c r="B55" s="66" t="s">
+      <c r="B55" s="70" t="s">
         <v>87</v>
       </c>
       <c r="C55" s="28" t="s">
@@ -3322,8 +3322,8 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="65"/>
-      <c r="B56" s="67"/>
+      <c r="A56" s="68"/>
+      <c r="B56" s="65"/>
       <c r="C56" s="13" t="s">
         <v>199</v>
       </c>
@@ -3336,13 +3336,13 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="65"/>
-      <c r="B57" s="69"/>
+      <c r="A57" s="68"/>
+      <c r="B57" s="66"/>
       <c r="E57" s="33"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="65"/>
-      <c r="B58" s="73" t="s">
+      <c r="A58" s="68"/>
+      <c r="B58" s="72" t="s">
         <v>6</v>
       </c>
       <c r="C58" s="37" t="s">
@@ -3357,8 +3357,8 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="65"/>
-      <c r="B59" s="70"/>
+      <c r="A59" s="68"/>
+      <c r="B59" s="73"/>
       <c r="C59" s="13" t="s">
         <v>135</v>
       </c>
@@ -3371,8 +3371,8 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="65"/>
-      <c r="B60" s="70"/>
+      <c r="A60" s="68"/>
+      <c r="B60" s="73"/>
       <c r="C60" s="13" t="s">
         <v>151</v>
       </c>
@@ -3385,8 +3385,8 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="65"/>
-      <c r="B61" s="70"/>
+      <c r="A61" s="68"/>
+      <c r="B61" s="73"/>
       <c r="C61" s="13" t="s">
         <v>183</v>
       </c>
@@ -3399,8 +3399,8 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="65"/>
-      <c r="B62" s="70"/>
+      <c r="A62" s="68"/>
+      <c r="B62" s="73"/>
       <c r="C62" s="13" t="s">
         <v>201</v>
       </c>
@@ -3413,8 +3413,8 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="65"/>
-      <c r="B63" s="70"/>
+      <c r="A63" s="68"/>
+      <c r="B63" s="73"/>
       <c r="C63" s="13" t="s">
         <v>209</v>
       </c>
@@ -3427,8 +3427,8 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="65"/>
-      <c r="B64" s="70"/>
+      <c r="A64" s="68"/>
+      <c r="B64" s="73"/>
       <c r="C64" s="13" t="s">
         <v>249</v>
       </c>
@@ -3441,8 +3441,8 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="65"/>
-      <c r="B65" s="70"/>
+      <c r="A65" s="68"/>
+      <c r="B65" s="73"/>
       <c r="C65" s="13" t="s">
         <v>215</v>
       </c>
@@ -3455,8 +3455,8 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="65"/>
-      <c r="B66" s="70"/>
+      <c r="A66" s="68"/>
+      <c r="B66" s="73"/>
       <c r="C66" s="13" t="s">
         <v>239</v>
       </c>
@@ -3469,12 +3469,12 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="65"/>
-      <c r="B67" s="75"/>
+      <c r="A67" s="68"/>
+      <c r="B67" s="74"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="65"/>
-      <c r="B68" s="73" t="s">
+      <c r="A68" s="68"/>
+      <c r="B68" s="72" t="s">
         <v>7</v>
       </c>
       <c r="C68" s="37" t="s">
@@ -3489,8 +3489,8 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="65"/>
-      <c r="B69" s="70"/>
+      <c r="A69" s="68"/>
+      <c r="B69" s="73"/>
       <c r="C69" s="13" t="s">
         <v>136</v>
       </c>
@@ -3503,8 +3503,8 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="65"/>
-      <c r="B70" s="70"/>
+      <c r="A70" s="68"/>
+      <c r="B70" s="73"/>
       <c r="C70" s="13" t="s">
         <v>149</v>
       </c>
@@ -3517,8 +3517,8 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="65"/>
-      <c r="B71" s="70"/>
+      <c r="A71" s="68"/>
+      <c r="B71" s="73"/>
       <c r="C71" s="13" t="s">
         <v>183</v>
       </c>
@@ -3531,8 +3531,8 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="65"/>
-      <c r="B72" s="70"/>
+      <c r="A72" s="68"/>
+      <c r="B72" s="73"/>
       <c r="C72" s="13" t="s">
         <v>201</v>
       </c>
@@ -3545,8 +3545,8 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="65"/>
-      <c r="B73" s="70"/>
+      <c r="A73" s="68"/>
+      <c r="B73" s="73"/>
       <c r="C73" s="13" t="s">
         <v>209</v>
       </c>
@@ -3559,8 +3559,8 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="65"/>
-      <c r="B74" s="70"/>
+      <c r="A74" s="68"/>
+      <c r="B74" s="73"/>
       <c r="C74" s="13" t="s">
         <v>249</v>
       </c>
@@ -3573,8 +3573,8 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="65"/>
-      <c r="B75" s="70"/>
+      <c r="A75" s="68"/>
+      <c r="B75" s="73"/>
       <c r="C75" s="13" t="s">
         <v>215</v>
       </c>
@@ -3587,8 +3587,8 @@
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="65"/>
-      <c r="B76" s="70"/>
+      <c r="A76" s="68"/>
+      <c r="B76" s="73"/>
       <c r="C76" s="13" t="s">
         <v>239</v>
       </c>
@@ -3602,13 +3602,13 @@
     </row>
     <row r="77" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="71"/>
-      <c r="B77" s="76"/>
+      <c r="B77" s="75"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="64" t="s">
+      <c r="A78" s="67" t="s">
         <v>90</v>
       </c>
-      <c r="B78" s="66" t="s">
+      <c r="B78" s="70" t="s">
         <v>87</v>
       </c>
       <c r="C78" s="28" t="s">
@@ -3623,8 +3623,8 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="65"/>
-      <c r="B79" s="67"/>
+      <c r="A79" s="68"/>
+      <c r="B79" s="65"/>
       <c r="C79" s="13" t="s">
         <v>291</v>
       </c>
@@ -3637,8 +3637,8 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="65"/>
-      <c r="B80" s="67"/>
+      <c r="A80" s="68"/>
+      <c r="B80" s="65"/>
       <c r="C80" s="13" t="s">
         <v>195</v>
       </c>
@@ -3651,13 +3651,13 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="65"/>
-      <c r="B81" s="69"/>
+      <c r="A81" s="68"/>
+      <c r="B81" s="66"/>
       <c r="E81" s="35"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="65"/>
-      <c r="B82" s="68" t="s">
+      <c r="A82" s="68"/>
+      <c r="B82" s="64" t="s">
         <v>93</v>
       </c>
       <c r="C82" s="37" t="s">
@@ -3672,8 +3672,8 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="65"/>
-      <c r="B83" s="67"/>
+      <c r="A83" s="68"/>
+      <c r="B83" s="65"/>
       <c r="C83" s="13" t="s">
         <v>196</v>
       </c>
@@ -3686,16 +3686,16 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="65"/>
-      <c r="B84" s="69"/>
+      <c r="A84" s="68"/>
+      <c r="B84" s="66"/>
       <c r="C84" s="39"/>
       <c r="D84" s="39"/>
       <c r="E84" s="40"/>
       <c r="F84" s="39"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="65"/>
-      <c r="B85" s="68" t="s">
+      <c r="A85" s="68"/>
+      <c r="B85" s="64" t="s">
         <v>94</v>
       </c>
       <c r="C85" s="13" t="s">
@@ -3710,8 +3710,8 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="65"/>
-      <c r="B86" s="67"/>
+      <c r="A86" s="68"/>
+      <c r="B86" s="65"/>
       <c r="C86" s="13" t="s">
         <v>197</v>
       </c>
@@ -3725,17 +3725,17 @@
     </row>
     <row r="87" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A87" s="71"/>
-      <c r="B87" s="74"/>
+      <c r="B87" s="69"/>
       <c r="C87" s="43"/>
       <c r="D87" s="43"/>
       <c r="E87" s="44"/>
       <c r="F87" s="43"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="64" t="s">
+      <c r="A88" s="67" t="s">
         <v>211</v>
       </c>
-      <c r="B88" s="66" t="s">
+      <c r="B88" s="70" t="s">
         <v>15</v>
       </c>
       <c r="C88" s="28" t="s">
@@ -3750,8 +3750,8 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="65"/>
-      <c r="B89" s="67"/>
+      <c r="A89" s="68"/>
+      <c r="B89" s="65"/>
       <c r="C89" s="13" t="s">
         <v>224</v>
       </c>
@@ -3763,16 +3763,16 @@
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="65"/>
-      <c r="B90" s="69"/>
+      <c r="A90" s="68"/>
+      <c r="B90" s="66"/>
       <c r="C90" s="39"/>
       <c r="D90" s="39"/>
       <c r="E90" s="39"/>
       <c r="F90" s="39"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="65"/>
-      <c r="B91" s="68" t="s">
+      <c r="A91" s="68"/>
+      <c r="B91" s="64" t="s">
         <v>234</v>
       </c>
       <c r="C91" s="13" t="s">
@@ -3786,8 +3786,8 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="65"/>
-      <c r="B92" s="67"/>
+      <c r="A92" s="68"/>
+      <c r="B92" s="65"/>
       <c r="C92" s="13" t="s">
         <v>232</v>
       </c>
@@ -3799,8 +3799,8 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="65"/>
-      <c r="B93" s="67"/>
+      <c r="A93" s="68"/>
+      <c r="B93" s="65"/>
       <c r="C93" s="13" t="s">
         <v>228</v>
       </c>
@@ -3812,8 +3812,8 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="65"/>
-      <c r="B94" s="67"/>
+      <c r="A94" s="68"/>
+      <c r="B94" s="65"/>
       <c r="C94" s="13" t="s">
         <v>230</v>
       </c>
@@ -3825,8 +3825,8 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="65"/>
-      <c r="B95" s="67"/>
+      <c r="A95" s="68"/>
+      <c r="B95" s="65"/>
       <c r="C95" s="13" t="s">
         <v>233</v>
       </c>
@@ -3838,8 +3838,8 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="65"/>
-      <c r="B96" s="67"/>
+      <c r="A96" s="68"/>
+      <c r="B96" s="65"/>
       <c r="C96" s="13" t="s">
         <v>242</v>
       </c>
@@ -3851,8 +3851,8 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="65"/>
-      <c r="B97" s="68" t="s">
+      <c r="A97" s="68"/>
+      <c r="B97" s="64" t="s">
         <v>263</v>
       </c>
       <c r="C97" s="37" t="s">
@@ -3867,8 +3867,8 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="65"/>
-      <c r="B98" s="67"/>
+      <c r="A98" s="68"/>
+      <c r="B98" s="65"/>
       <c r="C98" s="13" t="s">
         <v>259</v>
       </c>
@@ -3880,8 +3880,8 @@
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="65"/>
-      <c r="B99" s="67"/>
+      <c r="A99" s="68"/>
+      <c r="B99" s="65"/>
       <c r="C99" s="13" t="s">
         <v>274</v>
       </c>
@@ -3893,8 +3893,8 @@
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="65"/>
-      <c r="B100" s="67"/>
+      <c r="A100" s="68"/>
+      <c r="B100" s="65"/>
       <c r="C100" s="13" t="s">
         <v>260</v>
       </c>
@@ -3906,8 +3906,8 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="65"/>
-      <c r="B101" s="67"/>
+      <c r="A101" s="68"/>
+      <c r="B101" s="65"/>
       <c r="C101" s="13" t="s">
         <v>276</v>
       </c>
@@ -3919,8 +3919,8 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="65"/>
-      <c r="B102" s="67"/>
+      <c r="A102" s="68"/>
+      <c r="B102" s="65"/>
       <c r="C102" s="13" t="s">
         <v>280</v>
       </c>
@@ -3932,8 +3932,8 @@
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="65"/>
-      <c r="B103" s="67"/>
+      <c r="A103" s="68"/>
+      <c r="B103" s="65"/>
       <c r="C103" s="13" t="s">
         <v>257</v>
       </c>
@@ -3945,8 +3945,8 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="65"/>
-      <c r="B104" s="67"/>
+      <c r="A104" s="68"/>
+      <c r="B104" s="65"/>
       <c r="C104" s="13" t="s">
         <v>261</v>
       </c>
@@ -3958,8 +3958,8 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="65"/>
-      <c r="B105" s="67"/>
+      <c r="A105" s="68"/>
+      <c r="B105" s="65"/>
       <c r="C105" s="13" t="s">
         <v>262</v>
       </c>
@@ -3971,8 +3971,8 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="65"/>
-      <c r="B106" s="68" t="s">
+      <c r="A106" s="68"/>
+      <c r="B106" s="64" t="s">
         <v>281</v>
       </c>
       <c r="C106" s="37" t="s">
@@ -3987,8 +3987,8 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="65"/>
-      <c r="B107" s="67"/>
+      <c r="A107" s="68"/>
+      <c r="B107" s="65"/>
       <c r="C107" s="13" t="s">
         <v>284</v>
       </c>
@@ -4000,8 +4000,8 @@
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="65"/>
-      <c r="B108" s="67"/>
+      <c r="A108" s="68"/>
+      <c r="B108" s="65"/>
       <c r="C108" s="13" t="s">
         <v>286</v>
       </c>
@@ -4013,8 +4013,8 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="65"/>
-      <c r="B109" s="67"/>
+      <c r="A109" s="68"/>
+      <c r="B109" s="65"/>
       <c r="C109" s="13" t="s">
         <v>287</v>
       </c>
@@ -4026,12 +4026,12 @@
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="65"/>
-      <c r="B110" s="69"/>
+      <c r="A110" s="68"/>
+      <c r="B110" s="66"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="65"/>
-      <c r="B111" s="68" t="s">
+      <c r="A111" s="68"/>
+      <c r="B111" s="64" t="s">
         <v>292</v>
       </c>
       <c r="C111" s="37" t="s">
@@ -4046,8 +4046,8 @@
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="65"/>
-      <c r="B112" s="67"/>
+      <c r="A112" s="68"/>
+      <c r="B112" s="65"/>
       <c r="C112" s="13" t="s">
         <v>295</v>
       </c>
@@ -4060,6 +4060,13 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A2:A32"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B22"/>
+    <mergeCell ref="B23:B32"/>
+    <mergeCell ref="A33:A54"/>
+    <mergeCell ref="B33:B42"/>
+    <mergeCell ref="B43:B54"/>
     <mergeCell ref="B111:B112"/>
     <mergeCell ref="B106:B110"/>
     <mergeCell ref="A88:A112"/>
@@ -4074,13 +4081,6 @@
     <mergeCell ref="A78:A87"/>
     <mergeCell ref="B78:B81"/>
     <mergeCell ref="B82:B84"/>
-    <mergeCell ref="A2:A32"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B22"/>
-    <mergeCell ref="B23:B32"/>
-    <mergeCell ref="A33:A54"/>
-    <mergeCell ref="B33:B42"/>
-    <mergeCell ref="B43:B54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>